<commit_message>
1. Frontend updates based on user feedbacks and comments. 2. Database update: added a new Short description field for Products, Reagents, and Services.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/bioark-product-bulk-upload-template.xlsx
+++ b/frontend/public/templates/bioark-product-bulk-upload-template.xlsx
@@ -663,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -689,6 +689,7 @@
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
     <col width="21" customWidth="1" min="23" max="23"/>
+    <col width="38" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -807,10 +808,15 @@
           <t>display_order</t>
         </is>
       </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>short_description</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W1001"/>
-  <conditionalFormatting sqref="A2:W1001">
+  <autoFilter ref="A1:X1001"/>
+  <conditionalFormatting sqref="A2:X1001">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -851,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C40"/>
+  <dimension ref="B2:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1258,6 +1264,18 @@
       <c r="C40" s="13" t="inlineStr">
         <is>
           <t>Optional whole number used to order catalog entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>short_description</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Optional one-line customer-facing summary used on catalog display cards (maximum 500 characters).</t>
         </is>
       </c>
     </row>

</xml_diff>